<commit_message>
test(finance): close tax UI and export acceptance chain
</commit_message>
<xml_diff>
--- a/backend/tests/fixtures_t3_export/t3-report.xlsx
+++ b/backend/tests/fixtures_t3_export/t3-report.xlsx
@@ -456,7 +456,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>t3______4jkiqc</t>
+          <t>d3________vu05qt</t>
         </is>
       </c>
     </row>
@@ -516,7 +516,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>#337</t>
+          <t>#747</t>
         </is>
       </c>
     </row>
@@ -528,7 +528,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>#16</t>
+          <t>#22</t>
         </is>
       </c>
     </row>
@@ -551,7 +551,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>31</v>
+        <v>61</v>
       </c>
     </row>
     <row r="12">
@@ -632,7 +632,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>evidence_package=8, assessment=8</t>
+          <t>evidence_package=20, assessment=27</t>
         </is>
       </c>
     </row>
@@ -656,7 +656,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>系统自动评估(规则版本 1.0.0, 维度: physical, optimality, financial, reliability)</t>
         </is>
       </c>
     </row>
@@ -786,34 +786,34 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>load1</t>
+          <t>pv1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ies.device.electric_load</t>
+          <t>ies.device.pv</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>{"electricity_demand": 50, "peak_power_kw": 200}</t>
+          <t>{"ambient_temperature": 25, "rated_capacity_kwp": 100, "solar_irradiance": 500}</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>hp1</t>
+          <t>boiler1</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ies.device.heat_pump</t>
+          <t>ies.device.gas_boiler</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>{"cop": 3.5, "rated_heat_kw": 600}</t>
+          <t>{"lhv_kwh_per_m3": 9.97, "rated_heat_kw": 50, "thermal_efficiency": 0.9}</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>{"heat_demand": 30}</t>
+          <t>{"heat_demand": 10, "peak_heat_kw": 10}</t>
         </is>
       </c>
     </row>
@@ -845,7 +845,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B196"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -905,7 +905,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>tax_inclusive</t>
+          <t>tax_exclusive</t>
         </is>
       </c>
     </row>
@@ -937,7 +937,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>140000.0 CNY</t>
+          <t>677999.9999999999 CNY</t>
         </is>
       </c>
     </row>
@@ -949,7 +949,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0.6 × C = 84000.00 CNY</t>
+          <t>0.6 × C = 406799.99999999994 CNY</t>
         </is>
       </c>
     </row>
@@ -961,7 +961,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0.4 × C = 56000.00 CNY</t>
+          <t>0.4 × C = 271200.0 CNY</t>
         </is>
       </c>
     </row>
@@ -973,7 +973,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>能源 -359160.0 − 可变 600.6857142857142 − 固定 1400.0 − 维护 0 = 净额 -361160.6857142857142 CNY</t>
+          <t>能源 579079.7999999757 − 可变 0.0 − 固定 6360.0 − 维护 100 = 净额 572619.7999999756 CNY</t>
         </is>
       </c>
     </row>
@@ -985,7 +985,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>能源 -359160.0 − 可变 600.6857142857142 − 固定 1400.0 − 维护 3500.5 = 净额 -364661.1857142857142 CNY</t>
+          <t>能源 579079.7999999757 − 可变 0.0 − 固定 6360.0 − 维护 50 = 净额 572669.7999999757 CNY</t>
         </is>
       </c>
     </row>
@@ -997,7 +997,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>'-84000.00 CNY</t>
+          <t>'-406799.99999999994 CNY</t>
         </is>
       </c>
     </row>
@@ -1009,7 +1009,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>'-84000.00 / -84000.00 / -84000.00 CNY</t>
+          <t>'-406799.99999999994 / -406799.99999999994 / -406799.99999999994 CNY</t>
         </is>
       </c>
     </row>
@@ -1021,7 +1021,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>'-56000.00 CNY</t>
+          <t>'-271200.0 CNY</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1033,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>'-51851.85185185185185185185185 / -140000.00 / -135851.8518518518518518518518 CNY</t>
+          <t>'-251111.1111111111111111111111 / -677999.99999999994 / -657911.1111111110511111111111 CNY</t>
         </is>
       </c>
     </row>
@@ -1045,7 +1045,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>'-361160.6857142857142 CNY</t>
+          <t>454026.9238937746 CNY</t>
         </is>
       </c>
     </row>
@@ -1057,7 +1057,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>'-309637.0762296688221879286694 / -501160.6857142857142 / -445488.9280815206740397805212 CNY</t>
+          <t>389254.9073163362482853223594 / -223973.07610622534 / -268656.2037947748028257887517 CNY</t>
         </is>
       </c>
     </row>
@@ -1069,7 +1069,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>'-364661.1857142857142 CNY</t>
+          <t>397046.70442474395 CNY</t>
         </is>
       </c>
     </row>
@@ -1081,55 +1081,2095 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>'-289479.8062686437171353452218 / -865821.8714285714284 / -734968.7343501643911751257430 CNY</t>
+          <t>315188.4751631674144566377077 / 173073.62831851861 / 46532.2713683926116308489560 CNY</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>净现值 NPV / NPV</t>
+          <t>税后现金流 CF[t=0] / After-tax CF[t=0]</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>'-734968.7343501643911751257430 CNY</t>
+          <t>'-406799.99999999994 CNY</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>内部收益率 IRR / IRR</t>
+          <t>税后现金流 CF[t=1] / After-tax CF[t=1]</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>— / no_solution</t>
+          <t>'-271200.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>静态回收期 / static payback</t>
+          <t>税后现金流 CF[t=2] / After-tax CF[t=2]</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>— / not_recovered</t>
+          <t>454026.9238937746 CNY</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>税后现金流 CF[t=3] / After-tax CF[t=3]</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>397046.70442474395 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=1 / VAT main_pool m=1 实缴 / paid</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=1 / VAT main_pool m=1 确认退款 / claimed</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=1 / VAT main_pool m=1 到账退款 / arrived</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=1 / VAT main_pool m=1 期末结转 / carry</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>46800.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=2 / VAT main_pool m=2 实缴 / paid</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=2 / VAT main_pool m=2 确认退款 / claimed</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=2 / VAT main_pool m=2 到账退款 / arrived</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=2 / VAT main_pool m=2 期末结转 / carry</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>46800.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=3 / VAT main_pool m=3 实缴 / paid</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=3 / VAT main_pool m=3 确认退款 / claimed</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=3 / VAT main_pool m=3 到账退款 / arrived</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=3 / VAT main_pool m=3 期末结转 / carry</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>46800.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=4 / VAT main_pool m=4 实缴 / paid</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=4 / VAT main_pool m=4 确认退款 / claimed</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=4 / VAT main_pool m=4 到账退款 / arrived</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=4 / VAT main_pool m=4 期末结转 / carry</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>46800.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=5 / VAT main_pool m=5 实缴 / paid</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=5 / VAT main_pool m=5 确认退款 / claimed</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=5 / VAT main_pool m=5 到账退款 / arrived</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=5 / VAT main_pool m=5 期末结转 / carry</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>46800.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=6 / VAT main_pool m=6 实缴 / paid</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=6 / VAT main_pool m=6 确认退款 / claimed</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=6 / VAT main_pool m=6 到账退款 / arrived</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=6 / VAT main_pool m=6 期末结转 / carry</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>46800.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=7 / VAT main_pool m=7 实缴 / paid</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=7 / VAT main_pool m=7 确认退款 / claimed</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=7 / VAT main_pool m=7 到账退款 / arrived</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=7 / VAT main_pool m=7 期末结转 / carry</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>46800.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=8 / VAT main_pool m=8 实缴 / paid</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=8 / VAT main_pool m=8 确认退款 / claimed</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=8 / VAT main_pool m=8 到账退款 / arrived</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=8 / VAT main_pool m=8 期末结转 / carry</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>46800.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=9 / VAT main_pool m=9 实缴 / paid</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=9 / VAT main_pool m=9 确认退款 / claimed</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=9 / VAT main_pool m=9 到账退款 / arrived</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=9 / VAT main_pool m=9 期末结转 / carry</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>46800.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=10 / VAT main_pool m=10 实缴 / paid</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=10 / VAT main_pool m=10 确认退款 / claimed</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=10 / VAT main_pool m=10 到账退款 / arrived</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=10 / VAT main_pool m=10 期末结转 / carry</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>46800.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=11 / VAT main_pool m=11 实缴 / paid</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=11 / VAT main_pool m=11 确认退款 / claimed</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=11 / VAT main_pool m=11 到账退款 / arrived</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=11 / VAT main_pool m=11 期末结转 / carry</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>46800.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=12 / VAT main_pool m=12 实缴 / paid</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=12 / VAT main_pool m=12 确认退款 / claimed</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=12 / VAT main_pool m=12 到账退款 / arrived</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=12 / VAT main_pool m=12 期末结转 / carry</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>46800.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=13 / VAT main_pool m=13 实缴 / paid</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=13 / VAT main_pool m=13 确认退款 / claimed</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=13 / VAT main_pool m=13 到账退款 / arrived</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=13 / VAT main_pool m=13 期末结转 / carry</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>72341.87999999832 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=14 / VAT main_pool m=14 实缴 / paid</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=14 / VAT main_pool m=14 确认退款 / claimed</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>500.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=14 / VAT main_pool m=14 到账退款 / arrived</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=14 / VAT main_pool m=14 期末结转 / carry</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>66731.31999999823 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=15 / VAT main_pool m=15 实缴 / paid</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=15 / VAT main_pool m=15 确认退款 / claimed</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=15 / VAT main_pool m=15 到账退款 / arrived</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=15 / VAT main_pool m=15 期末结转 / carry</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>61073.19999999815 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=16 / VAT main_pool m=16 实缴 / paid</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=16 / VAT main_pool m=16 确认退款 / claimed</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=16 / VAT main_pool m=16 到账退款 / arrived</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>500.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=16 / VAT main_pool m=16 期末结转 / carry</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>55597.599999998056 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=17 / VAT main_pool m=17 实缴 / paid</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=17 / VAT main_pool m=17 确认退款 / claimed</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=17 / VAT main_pool m=17 到账退款 / arrived</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=17 / VAT main_pool m=17 期末结转 / carry</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>49939.479999997966 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=18 / VAT main_pool m=18 实缴 / paid</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=18 / VAT main_pool m=18 确认退款 / claimed</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=18 / VAT main_pool m=18 到账退款 / arrived</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=18 / VAT main_pool m=18 期末结转 / carry</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>44463.87999999788 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=19 / VAT main_pool m=19 实缴 / paid</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=19 / VAT main_pool m=19 确认退款 / claimed</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=19 / VAT main_pool m=19 到账退款 / arrived</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=19 / VAT main_pool m=19 期末结转 / carry</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>38805.75999999778 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=20 / VAT main_pool m=20 实缴 / paid</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=20 / VAT main_pool m=20 确认退款 / claimed</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>1500.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=20 / VAT main_pool m=20 到账退款 / arrived</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=20 / VAT main_pool m=20 期末结转 / carry</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>31647.639999997693 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=21 / VAT main_pool m=21 实缴 / paid</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=21 / VAT main_pool m=21 确认退款 / claimed</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=21 / VAT main_pool m=21 到账退款 / arrived</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=21 / VAT main_pool m=21 期末结转 / carry</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>26172.039999997563 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=22 / VAT main_pool m=22 实缴 / paid</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=22 / VAT main_pool m=22 确认退款 / claimed</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=22 / VAT main_pool m=22 到账退款 / arrived</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=22 / VAT main_pool m=22 期末结转 / carry</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>20513.91999999747 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=23 / VAT main_pool m=23 实缴 / paid</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=23 / VAT main_pool m=23 确认退款 / claimed</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=23 / VAT main_pool m=23 到账退款 / arrived</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=23 / VAT main_pool m=23 期末结转 / carry</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>15038.319999997382 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=24 / VAT main_pool m=24 实缴 / paid</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=24 / VAT main_pool m=24 确认退款 / claimed</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=24 / VAT main_pool m=24 到账退款 / arrived</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=24 / VAT main_pool m=24 期末结转 / carry</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>9751.704424776059 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=25 / VAT main_pool m=25 实缴 / paid</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=25 / VAT main_pool m=25 确认退款 / claimed</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=25 / VAT main_pool m=25 到账退款 / arrived</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=25 / VAT main_pool m=25 期末结转 / carry</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>4093.5844247759655 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=26 / VAT main_pool m=26 实缴 / paid</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>1016.9755752241139 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=26 / VAT main_pool m=26 确认退款 / claimed</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=26 / VAT main_pool m=26 到账退款 / arrived</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=26 / VAT main_pool m=26 期末结转 / carry</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=27 / VAT main_pool m=27 实缴 / paid</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>5658.120000000093 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=27 / VAT main_pool m=27 确认退款 / claimed</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=27 / VAT main_pool m=27 到账退款 / arrived</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=27 / VAT main_pool m=27 期末结转 / carry</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=28 / VAT main_pool m=28 实缴 / paid</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>5475.600000000089 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=28 / VAT main_pool m=28 确认退款 / claimed</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=28 / VAT main_pool m=28 到账退款 / arrived</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=28 / VAT main_pool m=28 期末结转 / carry</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=29 / VAT main_pool m=29 实缴 / paid</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>5658.120000000093 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=29 / VAT main_pool m=29 确认退款 / claimed</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=29 / VAT main_pool m=29 到账退款 / arrived</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=29 / VAT main_pool m=29 期末结转 / carry</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=30 / VAT main_pool m=30 实缴 / paid</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>5475.600000000089 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=30 / VAT main_pool m=30 确认退款 / claimed</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=30 / VAT main_pool m=30 到账退款 / arrived</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=30 / VAT main_pool m=30 期末结转 / carry</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=31 / VAT main_pool m=31 实缴 / paid</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>5658.120000000093 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=31 / VAT main_pool m=31 确认退款 / claimed</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=31 / VAT main_pool m=31 到账退款 / arrived</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=31 / VAT main_pool m=31 期末结转 / carry</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=32 / VAT main_pool m=32 实缴 / paid</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>5658.120000000093 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=32 / VAT main_pool m=32 确认退款 / claimed</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=32 / VAT main_pool m=32 到账退款 / arrived</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=32 / VAT main_pool m=32 期末结转 / carry</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=33 / VAT main_pool m=33 实缴 / paid</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>5475.600000000089 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=33 / VAT main_pool m=33 确认退款 / claimed</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=33 / VAT main_pool m=33 到账退款 / arrived</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=33 / VAT main_pool m=33 期末结转 / carry</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=34 / VAT main_pool m=34 实缴 / paid</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>5658.120000000093 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=34 / VAT main_pool m=34 确认退款 / claimed</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=34 / VAT main_pool m=34 到账退款 / arrived</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=34 / VAT main_pool m=34 期末结转 / carry</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=35 / VAT main_pool m=35 实缴 / paid</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>5475.600000000089 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=35 / VAT main_pool m=35 确认退款 / claimed</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=35 / VAT main_pool m=35 到账退款 / arrived</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=35 / VAT main_pool m=35 期末结转 / carry</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=36 / VAT main_pool m=36 实缴 / paid</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>5298.1200000000845 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=36 / VAT main_pool m=36 确认退款 / claimed</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=36 / VAT main_pool m=36 到账退款 / arrived</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>增值税 main_pool m=36 / VAT main_pool m=36 期末结转 / carry</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>退款 main_pool 确认m=14→到账m=16 / Refund main_pool confirm m=14→arrive m=16</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>500.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>退款 main_pool 确认m=20→到账m=40(期后应收，非期内现金) / Refund main_pool confirm m=20→arrive m=40</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>1500.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>所得税 income y=1 / Income income y=1 税基 / base</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>所得税 income y=1 / Income income y=1 抵亏 / used</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>所得税 income y=1 / Income income y=1 新生亏损 / generated</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>所得税 income y=1 / Income income y=1 到期核销 / expired</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>所得税 income y=1 / Income income y=1 税额 / tax</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>所得税 income y=2 / Income income y=2 税基 / base</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>476371.50442477874 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>所得税 income y=2 / Income income y=2 抵亏 / used</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>所得税 income y=2 / Income income y=2 新生亏损 / generated</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>所得税 income y=2 / Income income y=2 到期核销 / expired</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>所得税 income y=2 / Income income y=2 税额 / tax</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>119092.87610620132 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>所得税 income y=3 / Income income y=3 税基 / base</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>476460.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>所得税 income y=3 / Income income y=3 抵亏 / used</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>所得税 income y=3 / Income income y=3 新生亏损 / generated</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>所得税 income y=3 / Income income y=3 到期核销 / expired</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>所得税 income y=3 / Income income y=3 税额 / tax</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>119115.00000000664 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>计税折旧 income pv_system y=2 / Depreciation income pv_system y=2</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>30000.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>计税折旧 income pv_system y=3 / Depreciation income pv_system y=3</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>30000.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>亏损余额 income v0 y=2 (可用至y=7) / Loss balance</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>亏损余额 income v0 y=3 (可用至y=7) / Loss balance</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>亏损余额 income v1 y=3 (可用至y=8) / Loss balance</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>0.0 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>净现值 NPV / NPV</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>46532.2713683926116308489560 CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>内部收益率 IRR / IRR</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>0.11632899562309858 / normal</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>静态回收期 / static payback</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>2.564097557315646 year / recovered</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
           <t>动态回收期 / dynamic payback</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>— / not_recovered</t>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>2.8523668375110995 year / recovered</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test(finance): migrate exact XLSX seal fixture to evaluation 3.0.0
</commit_message>
<xml_diff>
--- a/backend/tests/fixtures_t3_export/t3-report.xlsx
+++ b/backend/tests/fixtures_t3_export/t3-report.xlsx
@@ -841,24 +841,20 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B196"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:B197"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>财务摘要 / Financial Summary</t>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">财务摘要 / Financial Summary</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>评价年限 E / Evaluation years</t>
+          <t xml:space="preserve">评价年限 E / Evaluation years</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -868,7 +864,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>建设期 K(财务时点 t=0..K) / Construction period</t>
+          <t xml:space="preserve">建设期 K(财务时点 t=0..K) / Construction period</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -878,7 +874,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>运营年限 N(第 j 年落 t=K+j) / Operation years</t>
+          <t xml:space="preserve">运营年限 N(第 j 年落 t=K+j) / Operation years</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -888,31 +884,31 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>币种 / Currency</t>
+          <t xml:space="preserve">币种 / Currency</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CNY</t>
+          <t xml:space="preserve">CNY</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>价格口径 / Price basis</t>
+          <t xml:space="preserve">价格口径 / Price basis</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>tax_exclusive</t>
+          <t xml:space="preserve">tax_exclusive</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>基年 / Base year</t>
+          <t xml:space="preserve">基年 / Base year</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -922,7 +918,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>折现率(冻结) / Discount rate</t>
+          <t xml:space="preserve">折现率(冻结) / Discount rate</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -932,2244 +928,2256 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>建设总额 C / Construction total</t>
+          <t xml:space="preserve">建设总额 C / Construction total</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>677999.9999999999 CNY</t>
+          <t xml:space="preserve">677999.9999999999 CNY</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>建设付款 t=0 / Payment t=0</t>
+          <t xml:space="preserve">建设付款 t=0 / Payment t=0</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0.6 × C = 406799.99999999994 CNY</t>
+          <t xml:space="preserve">0.6 × C = 406799.99999999994 CNY</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>建设付款 t=1 / Payment t=1</t>
+          <t xml:space="preserve">建设付款 t=1 / Payment t=1</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0.4 × C = 271200.0 CNY</t>
+          <t xml:space="preserve">0.4 × C = 271200.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>运营年第 1 年(t=2) / Year 1</t>
+          <t xml:space="preserve">运营年第 1 年(t=2) / Year 1</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>能源 579079.7999999757 − 可变 0.0 − 固定 6360.0 − 维护 100 = 净额 572619.7999999756 CNY</t>
+          <t xml:space="preserve">能源 579079.7999999757 − 可变 0.0 − 固定 6360.0 − 维护 100 − 需量 0.0 = 净额 572619.7999999756 CNY</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>运营年第 2 年(t=3) / Year 2</t>
+          <t xml:space="preserve">运营年第 2 年(t=3) / Year 2</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>能源 579079.7999999757 − 可变 0.0 − 固定 6360.0 − 维护 50 = 净额 572669.7999999757 CNY</t>
+          <t xml:space="preserve">能源 579079.7999999757 − 可变 0.0 − 固定 6360.0 − 维护 50 − 需量 0.0 = 净额 572669.7999999757 CNY</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CF[t=0] 净额 / Net</t>
+          <t xml:space="preserve">CF[t=0] 净额 / Net</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>'-406799.99999999994 CNY</t>
+          <t xml:space="preserve">'-406799.99999999994 CNY</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CF[t=0] 贴现/累计/贴现累计</t>
+          <t xml:space="preserve">CF[t=0] 贴现/累计/贴现累计</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>'-406799.99999999994 / -406799.99999999994 / -406799.99999999994 CNY</t>
+          <t xml:space="preserve">'-406799.99999999994 / -406799.99999999994 / -406799.99999999994 CNY</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CF[t=1] 净额 / Net</t>
+          <t xml:space="preserve">CF[t=1] 净额 / Net</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>'-271200.0 CNY</t>
+          <t xml:space="preserve">'-271200.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CF[t=1] 贴现/累计/贴现累计</t>
+          <t xml:space="preserve">CF[t=1] 贴现/累计/贴现累计</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>'-251111.1111111111111111111111 / -677999.99999999994 / -657911.1111111110511111111111 CNY</t>
+          <t xml:space="preserve">'-251111.1111111111111111111111 / -677999.99999999994 / -657911.1111111110511111111111 CNY</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CF[t=2] 净额 / Net</t>
+          <t xml:space="preserve">CF[t=2] 净额 / Net</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>454026.9238937746 CNY</t>
+          <t xml:space="preserve">454026.9238937746 CNY</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CF[t=2] 贴现/累计/贴现累计</t>
+          <t xml:space="preserve">CF[t=2] 贴现/累计/贴现累计</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>389254.9073163362482853223594 / -223973.07610622534 / -268656.2037947748028257887517 CNY</t>
+          <t xml:space="preserve">389254.9073163362482853223594 / -223973.07610622534 / -268656.2037947748028257887517 CNY</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CF[t=3] 净额 / Net</t>
+          <t xml:space="preserve">CF[t=3] 净额 / Net</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>397046.70442474395 CNY</t>
+          <t xml:space="preserve">397046.70442474395 CNY</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CF[t=3] 贴现/累计/贴现累计</t>
+          <t xml:space="preserve">CF[t=3] 贴现/累计/贴现累计</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>315188.4751631674144566377077 / 173073.62831851861 / 46532.2713683926116308489560 CNY</t>
+          <t xml:space="preserve">315188.4751631674144566377077 / 173073.62831851861 / 46532.2713683926116308489560 CNY</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>税后现金流 CF[t=0] / After-tax CF[t=0]</t>
+          <t xml:space="preserve">显式净现金 / Explicit net cashflows</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>'-406799.99999999994 CNY</t>
+          <t xml:space="preserve">无项目 / None</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>税后现金流 CF[t=1] / After-tax CF[t=1]</t>
+          <t xml:space="preserve">税后现金流 CF[t=0] / After-tax CF[t=0]</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>'-271200.0 CNY</t>
+          <t xml:space="preserve">'-406799.99999999994 CNY</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>税后现金流 CF[t=2] / After-tax CF[t=2]</t>
+          <t xml:space="preserve">税后现金流 CF[t=1] / After-tax CF[t=1]</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>454026.9238937746 CNY</t>
+          <t xml:space="preserve">'-271200.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>税后现金流 CF[t=3] / After-tax CF[t=3]</t>
+          <t xml:space="preserve">税后现金流 CF[t=2] / After-tax CF[t=2]</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>397046.70442474395 CNY</t>
+          <t xml:space="preserve">454026.9238937746 CNY</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=1 / VAT main_pool m=1 实缴 / paid</t>
+          <t xml:space="preserve">税后现金流 CF[t=3] / After-tax CF[t=3]</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">397046.70442474395 CNY</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=1 / VAT main_pool m=1 确认退款 / claimed</t>
+          <t xml:space="preserve">增值税 main_pool m=1 / VAT main_pool m=1 实缴 / paid</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=1 / VAT main_pool m=1 到账退款 / arrived</t>
+          <t xml:space="preserve">增值税 main_pool m=1 / VAT main_pool m=1 确认退款 / claimed</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=1 / VAT main_pool m=1 期末结转 / carry</t>
+          <t xml:space="preserve">增值税 main_pool m=1 / VAT main_pool m=1 到账退款 / arrived</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>46800.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=2 / VAT main_pool m=2 实缴 / paid</t>
+          <t xml:space="preserve">增值税 main_pool m=1 / VAT main_pool m=1 期末结转 / carry</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">46800.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=2 / VAT main_pool m=2 确认退款 / claimed</t>
+          <t xml:space="preserve">增值税 main_pool m=2 / VAT main_pool m=2 实缴 / paid</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=2 / VAT main_pool m=2 到账退款 / arrived</t>
+          <t xml:space="preserve">增值税 main_pool m=2 / VAT main_pool m=2 确认退款 / claimed</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=2 / VAT main_pool m=2 期末结转 / carry</t>
+          <t xml:space="preserve">增值税 main_pool m=2 / VAT main_pool m=2 到账退款 / arrived</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>46800.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=3 / VAT main_pool m=3 实缴 / paid</t>
+          <t xml:space="preserve">增值税 main_pool m=2 / VAT main_pool m=2 期末结转 / carry</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">46800.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=3 / VAT main_pool m=3 确认退款 / claimed</t>
+          <t xml:space="preserve">增值税 main_pool m=3 / VAT main_pool m=3 实缴 / paid</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=3 / VAT main_pool m=3 到账退款 / arrived</t>
+          <t xml:space="preserve">增值税 main_pool m=3 / VAT main_pool m=3 确认退款 / claimed</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=3 / VAT main_pool m=3 期末结转 / carry</t>
+          <t xml:space="preserve">增值税 main_pool m=3 / VAT main_pool m=3 到账退款 / arrived</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>46800.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=4 / VAT main_pool m=4 实缴 / paid</t>
+          <t xml:space="preserve">增值税 main_pool m=3 / VAT main_pool m=3 期末结转 / carry</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">46800.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=4 / VAT main_pool m=4 确认退款 / claimed</t>
+          <t xml:space="preserve">增值税 main_pool m=4 / VAT main_pool m=4 实缴 / paid</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=4 / VAT main_pool m=4 到账退款 / arrived</t>
+          <t xml:space="preserve">增值税 main_pool m=4 / VAT main_pool m=4 确认退款 / claimed</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=4 / VAT main_pool m=4 期末结转 / carry</t>
+          <t xml:space="preserve">增值税 main_pool m=4 / VAT main_pool m=4 到账退款 / arrived</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>46800.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=5 / VAT main_pool m=5 实缴 / paid</t>
+          <t xml:space="preserve">增值税 main_pool m=4 / VAT main_pool m=4 期末结转 / carry</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">46800.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=5 / VAT main_pool m=5 确认退款 / claimed</t>
+          <t xml:space="preserve">增值税 main_pool m=5 / VAT main_pool m=5 实缴 / paid</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=5 / VAT main_pool m=5 到账退款 / arrived</t>
+          <t xml:space="preserve">增值税 main_pool m=5 / VAT main_pool m=5 确认退款 / claimed</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=5 / VAT main_pool m=5 期末结转 / carry</t>
+          <t xml:space="preserve">增值税 main_pool m=5 / VAT main_pool m=5 到账退款 / arrived</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>46800.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=6 / VAT main_pool m=6 实缴 / paid</t>
+          <t xml:space="preserve">增值税 main_pool m=5 / VAT main_pool m=5 期末结转 / carry</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">46800.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=6 / VAT main_pool m=6 确认退款 / claimed</t>
+          <t xml:space="preserve">增值税 main_pool m=6 / VAT main_pool m=6 实缴 / paid</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=6 / VAT main_pool m=6 到账退款 / arrived</t>
+          <t xml:space="preserve">增值税 main_pool m=6 / VAT main_pool m=6 确认退款 / claimed</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=6 / VAT main_pool m=6 期末结转 / carry</t>
+          <t xml:space="preserve">增值税 main_pool m=6 / VAT main_pool m=6 到账退款 / arrived</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>46800.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=7 / VAT main_pool m=7 实缴 / paid</t>
+          <t xml:space="preserve">增值税 main_pool m=6 / VAT main_pool m=6 期末结转 / carry</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">46800.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=7 / VAT main_pool m=7 确认退款 / claimed</t>
+          <t xml:space="preserve">增值税 main_pool m=7 / VAT main_pool m=7 实缴 / paid</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=7 / VAT main_pool m=7 到账退款 / arrived</t>
+          <t xml:space="preserve">增值税 main_pool m=7 / VAT main_pool m=7 确认退款 / claimed</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=7 / VAT main_pool m=7 期末结转 / carry</t>
+          <t xml:space="preserve">增值税 main_pool m=7 / VAT main_pool m=7 到账退款 / arrived</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>46800.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=8 / VAT main_pool m=8 实缴 / paid</t>
+          <t xml:space="preserve">增值税 main_pool m=7 / VAT main_pool m=7 期末结转 / carry</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">46800.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=8 / VAT main_pool m=8 确认退款 / claimed</t>
+          <t xml:space="preserve">增值税 main_pool m=8 / VAT main_pool m=8 实缴 / paid</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=8 / VAT main_pool m=8 到账退款 / arrived</t>
+          <t xml:space="preserve">增值税 main_pool m=8 / VAT main_pool m=8 确认退款 / claimed</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=8 / VAT main_pool m=8 期末结转 / carry</t>
+          <t xml:space="preserve">增值税 main_pool m=8 / VAT main_pool m=8 到账退款 / arrived</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>46800.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=9 / VAT main_pool m=9 实缴 / paid</t>
+          <t xml:space="preserve">增值税 main_pool m=8 / VAT main_pool m=8 期末结转 / carry</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">46800.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=9 / VAT main_pool m=9 确认退款 / claimed</t>
+          <t xml:space="preserve">增值税 main_pool m=9 / VAT main_pool m=9 实缴 / paid</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=9 / VAT main_pool m=9 到账退款 / arrived</t>
+          <t xml:space="preserve">增值税 main_pool m=9 / VAT main_pool m=9 确认退款 / claimed</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=9 / VAT main_pool m=9 期末结转 / carry</t>
+          <t xml:space="preserve">增值税 main_pool m=9 / VAT main_pool m=9 到账退款 / arrived</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>46800.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=10 / VAT main_pool m=10 实缴 / paid</t>
+          <t xml:space="preserve">增值税 main_pool m=9 / VAT main_pool m=9 期末结转 / carry</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">46800.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=10 / VAT main_pool m=10 确认退款 / claimed</t>
+          <t xml:space="preserve">增值税 main_pool m=10 / VAT main_pool m=10 实缴 / paid</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=10 / VAT main_pool m=10 到账退款 / arrived</t>
+          <t xml:space="preserve">增值税 main_pool m=10 / VAT main_pool m=10 确认退款 / claimed</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=10 / VAT main_pool m=10 期末结转 / carry</t>
+          <t xml:space="preserve">增值税 main_pool m=10 / VAT main_pool m=10 到账退款 / arrived</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>46800.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=11 / VAT main_pool m=11 实缴 / paid</t>
+          <t xml:space="preserve">增值税 main_pool m=10 / VAT main_pool m=10 期末结转 / carry</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">46800.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=11 / VAT main_pool m=11 确认退款 / claimed</t>
+          <t xml:space="preserve">增值税 main_pool m=11 / VAT main_pool m=11 实缴 / paid</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=11 / VAT main_pool m=11 到账退款 / arrived</t>
+          <t xml:space="preserve">增值税 main_pool m=11 / VAT main_pool m=11 确认退款 / claimed</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=11 / VAT main_pool m=11 期末结转 / carry</t>
+          <t xml:space="preserve">增值税 main_pool m=11 / VAT main_pool m=11 到账退款 / arrived</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>46800.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=12 / VAT main_pool m=12 实缴 / paid</t>
+          <t xml:space="preserve">增值税 main_pool m=11 / VAT main_pool m=11 期末结转 / carry</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">46800.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=12 / VAT main_pool m=12 确认退款 / claimed</t>
+          <t xml:space="preserve">增值税 main_pool m=12 / VAT main_pool m=12 实缴 / paid</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=12 / VAT main_pool m=12 到账退款 / arrived</t>
+          <t xml:space="preserve">增值税 main_pool m=12 / VAT main_pool m=12 确认退款 / claimed</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=12 / VAT main_pool m=12 期末结转 / carry</t>
+          <t xml:space="preserve">增值税 main_pool m=12 / VAT main_pool m=12 到账退款 / arrived</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>46800.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=13 / VAT main_pool m=13 实缴 / paid</t>
+          <t xml:space="preserve">增值税 main_pool m=12 / VAT main_pool m=12 期末结转 / carry</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">46800.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=13 / VAT main_pool m=13 确认退款 / claimed</t>
+          <t xml:space="preserve">增值税 main_pool m=13 / VAT main_pool m=13 实缴 / paid</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=13 / VAT main_pool m=13 到账退款 / arrived</t>
+          <t xml:space="preserve">增值税 main_pool m=13 / VAT main_pool m=13 确认退款 / claimed</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=13 / VAT main_pool m=13 期末结转 / carry</t>
+          <t xml:space="preserve">增值税 main_pool m=13 / VAT main_pool m=13 到账退款 / arrived</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>72341.87999999832 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=14 / VAT main_pool m=14 实缴 / paid</t>
+          <t xml:space="preserve">增值税 main_pool m=13 / VAT main_pool m=13 期末结转 / carry</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">72341.87999999832 CNY</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=14 / VAT main_pool m=14 确认退款 / claimed</t>
+          <t xml:space="preserve">增值税 main_pool m=14 / VAT main_pool m=14 实缴 / paid</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>500.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=14 / VAT main_pool m=14 到账退款 / arrived</t>
+          <t xml:space="preserve">增值税 main_pool m=14 / VAT main_pool m=14 确认退款 / claimed</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">500.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=14 / VAT main_pool m=14 期末结转 / carry</t>
+          <t xml:space="preserve">增值税 main_pool m=14 / VAT main_pool m=14 到账退款 / arrived</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>66731.31999999823 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=15 / VAT main_pool m=15 实缴 / paid</t>
+          <t xml:space="preserve">增值税 main_pool m=14 / VAT main_pool m=14 期末结转 / carry</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">66731.31999999823 CNY</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=15 / VAT main_pool m=15 确认退款 / claimed</t>
+          <t xml:space="preserve">增值税 main_pool m=15 / VAT main_pool m=15 实缴 / paid</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=15 / VAT main_pool m=15 到账退款 / arrived</t>
+          <t xml:space="preserve">增值税 main_pool m=15 / VAT main_pool m=15 确认退款 / claimed</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=15 / VAT main_pool m=15 期末结转 / carry</t>
+          <t xml:space="preserve">增值税 main_pool m=15 / VAT main_pool m=15 到账退款 / arrived</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>61073.19999999815 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=16 / VAT main_pool m=16 实缴 / paid</t>
+          <t xml:space="preserve">增值税 main_pool m=15 / VAT main_pool m=15 期末结转 / carry</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">61073.19999999815 CNY</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=16 / VAT main_pool m=16 确认退款 / claimed</t>
+          <t xml:space="preserve">增值税 main_pool m=16 / VAT main_pool m=16 实缴 / paid</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=16 / VAT main_pool m=16 到账退款 / arrived</t>
+          <t xml:space="preserve">增值税 main_pool m=16 / VAT main_pool m=16 确认退款 / claimed</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>500.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=16 / VAT main_pool m=16 期末结转 / carry</t>
+          <t xml:space="preserve">增值税 main_pool m=16 / VAT main_pool m=16 到账退款 / arrived</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>55597.599999998056 CNY</t>
+          <t xml:space="preserve">500.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=17 / VAT main_pool m=17 实缴 / paid</t>
+          <t xml:space="preserve">增值税 main_pool m=16 / VAT main_pool m=16 期末结转 / carry</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">55597.599999998056 CNY</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=17 / VAT main_pool m=17 确认退款 / claimed</t>
+          <t xml:space="preserve">增值税 main_pool m=17 / VAT main_pool m=17 实缴 / paid</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=17 / VAT main_pool m=17 到账退款 / arrived</t>
+          <t xml:space="preserve">增值税 main_pool m=17 / VAT main_pool m=17 确认退款 / claimed</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=17 / VAT main_pool m=17 期末结转 / carry</t>
+          <t xml:space="preserve">增值税 main_pool m=17 / VAT main_pool m=17 到账退款 / arrived</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>49939.479999997966 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=18 / VAT main_pool m=18 实缴 / paid</t>
+          <t xml:space="preserve">增值税 main_pool m=17 / VAT main_pool m=17 期末结转 / carry</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">49939.479999997966 CNY</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=18 / VAT main_pool m=18 确认退款 / claimed</t>
+          <t xml:space="preserve">增值税 main_pool m=18 / VAT main_pool m=18 实缴 / paid</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=18 / VAT main_pool m=18 到账退款 / arrived</t>
+          <t xml:space="preserve">增值税 main_pool m=18 / VAT main_pool m=18 确认退款 / claimed</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=18 / VAT main_pool m=18 期末结转 / carry</t>
+          <t xml:space="preserve">增值税 main_pool m=18 / VAT main_pool m=18 到账退款 / arrived</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>44463.87999999788 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=19 / VAT main_pool m=19 实缴 / paid</t>
+          <t xml:space="preserve">增值税 main_pool m=18 / VAT main_pool m=18 期末结转 / carry</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">44463.87999999788 CNY</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=19 / VAT main_pool m=19 确认退款 / claimed</t>
+          <t xml:space="preserve">增值税 main_pool m=19 / VAT main_pool m=19 实缴 / paid</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=19 / VAT main_pool m=19 到账退款 / arrived</t>
+          <t xml:space="preserve">增值税 main_pool m=19 / VAT main_pool m=19 确认退款 / claimed</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=19 / VAT main_pool m=19 期末结转 / carry</t>
+          <t xml:space="preserve">增值税 main_pool m=19 / VAT main_pool m=19 到账退款 / arrived</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>38805.75999999778 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=20 / VAT main_pool m=20 实缴 / paid</t>
+          <t xml:space="preserve">增值税 main_pool m=19 / VAT main_pool m=19 期末结转 / carry</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">38805.75999999778 CNY</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=20 / VAT main_pool m=20 确认退款 / claimed</t>
+          <t xml:space="preserve">增值税 main_pool m=20 / VAT main_pool m=20 实缴 / paid</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>1500.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=20 / VAT main_pool m=20 到账退款 / arrived</t>
+          <t xml:space="preserve">增值税 main_pool m=20 / VAT main_pool m=20 确认退款 / claimed</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">1500.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=20 / VAT main_pool m=20 期末结转 / carry</t>
+          <t xml:space="preserve">增值税 main_pool m=20 / VAT main_pool m=20 到账退款 / arrived</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>31647.639999997693 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=21 / VAT main_pool m=21 实缴 / paid</t>
+          <t xml:space="preserve">增值税 main_pool m=20 / VAT main_pool m=20 期末结转 / carry</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">31647.639999997693 CNY</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=21 / VAT main_pool m=21 确认退款 / claimed</t>
+          <t xml:space="preserve">增值税 main_pool m=21 / VAT main_pool m=21 实缴 / paid</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=21 / VAT main_pool m=21 到账退款 / arrived</t>
+          <t xml:space="preserve">增值税 main_pool m=21 / VAT main_pool m=21 确认退款 / claimed</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=21 / VAT main_pool m=21 期末结转 / carry</t>
+          <t xml:space="preserve">增值税 main_pool m=21 / VAT main_pool m=21 到账退款 / arrived</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>26172.039999997563 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=22 / VAT main_pool m=22 实缴 / paid</t>
+          <t xml:space="preserve">增值税 main_pool m=21 / VAT main_pool m=21 期末结转 / carry</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">26172.039999997563 CNY</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=22 / VAT main_pool m=22 确认退款 / claimed</t>
+          <t xml:space="preserve">增值税 main_pool m=22 / VAT main_pool m=22 实缴 / paid</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=22 / VAT main_pool m=22 到账退款 / arrived</t>
+          <t xml:space="preserve">增值税 main_pool m=22 / VAT main_pool m=22 确认退款 / claimed</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=22 / VAT main_pool m=22 期末结转 / carry</t>
+          <t xml:space="preserve">增值税 main_pool m=22 / VAT main_pool m=22 到账退款 / arrived</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>20513.91999999747 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=23 / VAT main_pool m=23 实缴 / paid</t>
+          <t xml:space="preserve">增值税 main_pool m=22 / VAT main_pool m=22 期末结转 / carry</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">20513.91999999747 CNY</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=23 / VAT main_pool m=23 确认退款 / claimed</t>
+          <t xml:space="preserve">增值税 main_pool m=23 / VAT main_pool m=23 实缴 / paid</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=23 / VAT main_pool m=23 到账退款 / arrived</t>
+          <t xml:space="preserve">增值税 main_pool m=23 / VAT main_pool m=23 确认退款 / claimed</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=23 / VAT main_pool m=23 期末结转 / carry</t>
+          <t xml:space="preserve">增值税 main_pool m=23 / VAT main_pool m=23 到账退款 / arrived</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>15038.319999997382 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=24 / VAT main_pool m=24 实缴 / paid</t>
+          <t xml:space="preserve">增值税 main_pool m=23 / VAT main_pool m=23 期末结转 / carry</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">15038.319999997382 CNY</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=24 / VAT main_pool m=24 确认退款 / claimed</t>
+          <t xml:space="preserve">增值税 main_pool m=24 / VAT main_pool m=24 实缴 / paid</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=24 / VAT main_pool m=24 到账退款 / arrived</t>
+          <t xml:space="preserve">增值税 main_pool m=24 / VAT main_pool m=24 确认退款 / claimed</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=24 / VAT main_pool m=24 期末结转 / carry</t>
+          <t xml:space="preserve">增值税 main_pool m=24 / VAT main_pool m=24 到账退款 / arrived</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>9751.704424776059 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=25 / VAT main_pool m=25 实缴 / paid</t>
+          <t xml:space="preserve">增值税 main_pool m=24 / VAT main_pool m=24 期末结转 / carry</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">9751.704424776059 CNY</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=25 / VAT main_pool m=25 确认退款 / claimed</t>
+          <t xml:space="preserve">增值税 main_pool m=25 / VAT main_pool m=25 实缴 / paid</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=25 / VAT main_pool m=25 到账退款 / arrived</t>
+          <t xml:space="preserve">增值税 main_pool m=25 / VAT main_pool m=25 确认退款 / claimed</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=25 / VAT main_pool m=25 期末结转 / carry</t>
+          <t xml:space="preserve">增值税 main_pool m=25 / VAT main_pool m=25 到账退款 / arrived</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>4093.5844247759655 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=26 / VAT main_pool m=26 实缴 / paid</t>
+          <t xml:space="preserve">增值税 main_pool m=25 / VAT main_pool m=25 期末结转 / carry</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>1016.9755752241139 CNY</t>
+          <t xml:space="preserve">4093.5844247759655 CNY</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=26 / VAT main_pool m=26 确认退款 / claimed</t>
+          <t xml:space="preserve">增值税 main_pool m=26 / VAT main_pool m=26 实缴 / paid</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">1016.9755752241139 CNY</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=26 / VAT main_pool m=26 到账退款 / arrived</t>
+          <t xml:space="preserve">增值税 main_pool m=26 / VAT main_pool m=26 确认退款 / claimed</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=26 / VAT main_pool m=26 期末结转 / carry</t>
+          <t xml:space="preserve">增值税 main_pool m=26 / VAT main_pool m=26 到账退款 / arrived</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=27 / VAT main_pool m=27 实缴 / paid</t>
+          <t xml:space="preserve">增值税 main_pool m=26 / VAT main_pool m=26 期末结转 / carry</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>5658.120000000093 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=27 / VAT main_pool m=27 确认退款 / claimed</t>
+          <t xml:space="preserve">增值税 main_pool m=27 / VAT main_pool m=27 实缴 / paid</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">5658.120000000093 CNY</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=27 / VAT main_pool m=27 到账退款 / arrived</t>
+          <t xml:space="preserve">增值税 main_pool m=27 / VAT main_pool m=27 确认退款 / claimed</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=27 / VAT main_pool m=27 期末结转 / carry</t>
+          <t xml:space="preserve">增值税 main_pool m=27 / VAT main_pool m=27 到账退款 / arrived</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=28 / VAT main_pool m=28 实缴 / paid</t>
+          <t xml:space="preserve">增值税 main_pool m=27 / VAT main_pool m=27 期末结转 / carry</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>5475.600000000089 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=28 / VAT main_pool m=28 确认退款 / claimed</t>
+          <t xml:space="preserve">增值税 main_pool m=28 / VAT main_pool m=28 实缴 / paid</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">5475.600000000089 CNY</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=28 / VAT main_pool m=28 到账退款 / arrived</t>
+          <t xml:space="preserve">增值税 main_pool m=28 / VAT main_pool m=28 确认退款 / claimed</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=28 / VAT main_pool m=28 期末结转 / carry</t>
+          <t xml:space="preserve">增值税 main_pool m=28 / VAT main_pool m=28 到账退款 / arrived</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=29 / VAT main_pool m=29 实缴 / paid</t>
+          <t xml:space="preserve">增值税 main_pool m=28 / VAT main_pool m=28 期末结转 / carry</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>5658.120000000093 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=29 / VAT main_pool m=29 确认退款 / claimed</t>
+          <t xml:space="preserve">增值税 main_pool m=29 / VAT main_pool m=29 实缴 / paid</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">5658.120000000093 CNY</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=29 / VAT main_pool m=29 到账退款 / arrived</t>
+          <t xml:space="preserve">增值税 main_pool m=29 / VAT main_pool m=29 确认退款 / claimed</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=29 / VAT main_pool m=29 期末结转 / carry</t>
+          <t xml:space="preserve">增值税 main_pool m=29 / VAT main_pool m=29 到账退款 / arrived</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=30 / VAT main_pool m=30 实缴 / paid</t>
+          <t xml:space="preserve">增值税 main_pool m=29 / VAT main_pool m=29 期末结转 / carry</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>5475.600000000089 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=30 / VAT main_pool m=30 确认退款 / claimed</t>
+          <t xml:space="preserve">增值税 main_pool m=30 / VAT main_pool m=30 实缴 / paid</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">5475.600000000089 CNY</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=30 / VAT main_pool m=30 到账退款 / arrived</t>
+          <t xml:space="preserve">增值税 main_pool m=30 / VAT main_pool m=30 确认退款 / claimed</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=30 / VAT main_pool m=30 期末结转 / carry</t>
+          <t xml:space="preserve">增值税 main_pool m=30 / VAT main_pool m=30 到账退款 / arrived</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=31 / VAT main_pool m=31 实缴 / paid</t>
+          <t xml:space="preserve">增值税 main_pool m=30 / VAT main_pool m=30 期末结转 / carry</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>5658.120000000093 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=31 / VAT main_pool m=31 确认退款 / claimed</t>
+          <t xml:space="preserve">增值税 main_pool m=31 / VAT main_pool m=31 实缴 / paid</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">5658.120000000093 CNY</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=31 / VAT main_pool m=31 到账退款 / arrived</t>
+          <t xml:space="preserve">增值税 main_pool m=31 / VAT main_pool m=31 确认退款 / claimed</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=31 / VAT main_pool m=31 期末结转 / carry</t>
+          <t xml:space="preserve">增值税 main_pool m=31 / VAT main_pool m=31 到账退款 / arrived</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=32 / VAT main_pool m=32 实缴 / paid</t>
+          <t xml:space="preserve">增值税 main_pool m=31 / VAT main_pool m=31 期末结转 / carry</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>5658.120000000093 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=32 / VAT main_pool m=32 确认退款 / claimed</t>
+          <t xml:space="preserve">增值税 main_pool m=32 / VAT main_pool m=32 实缴 / paid</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">5658.120000000093 CNY</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=32 / VAT main_pool m=32 到账退款 / arrived</t>
+          <t xml:space="preserve">增值税 main_pool m=32 / VAT main_pool m=32 确认退款 / claimed</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=32 / VAT main_pool m=32 期末结转 / carry</t>
+          <t xml:space="preserve">增值税 main_pool m=32 / VAT main_pool m=32 到账退款 / arrived</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=33 / VAT main_pool m=33 实缴 / paid</t>
+          <t xml:space="preserve">增值税 main_pool m=32 / VAT main_pool m=32 期末结转 / carry</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>5475.600000000089 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=33 / VAT main_pool m=33 确认退款 / claimed</t>
+          <t xml:space="preserve">增值税 main_pool m=33 / VAT main_pool m=33 实缴 / paid</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">5475.600000000089 CNY</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=33 / VAT main_pool m=33 到账退款 / arrived</t>
+          <t xml:space="preserve">增值税 main_pool m=33 / VAT main_pool m=33 确认退款 / claimed</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=33 / VAT main_pool m=33 期末结转 / carry</t>
+          <t xml:space="preserve">增值税 main_pool m=33 / VAT main_pool m=33 到账退款 / arrived</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=34 / VAT main_pool m=34 实缴 / paid</t>
+          <t xml:space="preserve">增值税 main_pool m=33 / VAT main_pool m=33 期末结转 / carry</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>5658.120000000093 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=34 / VAT main_pool m=34 确认退款 / claimed</t>
+          <t xml:space="preserve">增值税 main_pool m=34 / VAT main_pool m=34 实缴 / paid</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">5658.120000000093 CNY</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=34 / VAT main_pool m=34 到账退款 / arrived</t>
+          <t xml:space="preserve">增值税 main_pool m=34 / VAT main_pool m=34 确认退款 / claimed</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=34 / VAT main_pool m=34 期末结转 / carry</t>
+          <t xml:space="preserve">增值税 main_pool m=34 / VAT main_pool m=34 到账退款 / arrived</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=35 / VAT main_pool m=35 实缴 / paid</t>
+          <t xml:space="preserve">增值税 main_pool m=34 / VAT main_pool m=34 期末结转 / carry</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>5475.600000000089 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=35 / VAT main_pool m=35 确认退款 / claimed</t>
+          <t xml:space="preserve">增值税 main_pool m=35 / VAT main_pool m=35 实缴 / paid</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">5475.600000000089 CNY</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=35 / VAT main_pool m=35 到账退款 / arrived</t>
+          <t xml:space="preserve">增值税 main_pool m=35 / VAT main_pool m=35 确认退款 / claimed</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=35 / VAT main_pool m=35 期末结转 / carry</t>
+          <t xml:space="preserve">增值税 main_pool m=35 / VAT main_pool m=35 到账退款 / arrived</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=36 / VAT main_pool m=36 实缴 / paid</t>
+          <t xml:space="preserve">增值税 main_pool m=35 / VAT main_pool m=35 期末结转 / carry</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>5298.1200000000845 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=36 / VAT main_pool m=36 确认退款 / claimed</t>
+          <t xml:space="preserve">增值税 main_pool m=36 / VAT main_pool m=36 实缴 / paid</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">5298.1200000000845 CNY</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=36 / VAT main_pool m=36 到账退款 / arrived</t>
+          <t xml:space="preserve">增值税 main_pool m=36 / VAT main_pool m=36 确认退款 / claimed</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>增值税 main_pool m=36 / VAT main_pool m=36 期末结转 / carry</t>
+          <t xml:space="preserve">增值税 main_pool m=36 / VAT main_pool m=36 到账退款 / arrived</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>退款 main_pool 确认m=14→到账m=16 / Refund main_pool confirm m=14→arrive m=16</t>
+          <t xml:space="preserve">增值税 main_pool m=36 / VAT main_pool m=36 期末结转 / carry</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>500.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>退款 main_pool 确认m=20→到账m=40(期后应收，非期内现金) / Refund main_pool confirm m=20→arrive m=40</t>
+          <t xml:space="preserve">退款 main_pool 确认m=14→到账m=16 / Refund main_pool confirm m=14→arrive m=16</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>1500.0 CNY</t>
+          <t xml:space="preserve">500.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>所得税 income y=1 / Income income y=1 税基 / base</t>
+          <t xml:space="preserve">退款 main_pool 确认m=20→到账m=40(期后应收，非期内现金) / Refund main_pool confirm m=20→arrive m=40</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">1500.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>所得税 income y=1 / Income income y=1 抵亏 / used</t>
+          <t xml:space="preserve">所得税 income y=1 / Income income y=1 税基 / base</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>所得税 income y=1 / Income income y=1 新生亏损 / generated</t>
+          <t xml:space="preserve">所得税 income y=1 / Income income y=1 抵亏 / used</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>所得税 income y=1 / Income income y=1 到期核销 / expired</t>
+          <t xml:space="preserve">所得税 income y=1 / Income income y=1 新生亏损 / generated</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>所得税 income y=1 / Income income y=1 税额 / tax</t>
+          <t xml:space="preserve">所得税 income y=1 / Income income y=1 到期核销 / expired</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>所得税 income y=2 / Income income y=2 税基 / base</t>
+          <t xml:space="preserve">所得税 income y=1 / Income income y=1 税额 / tax</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>476371.50442477874 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>所得税 income y=2 / Income income y=2 抵亏 / used</t>
+          <t xml:space="preserve">所得税 income y=2 / Income income y=2 税基 / base</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">476371.50442477874 CNY</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>所得税 income y=2 / Income income y=2 新生亏损 / generated</t>
+          <t xml:space="preserve">所得税 income y=2 / Income income y=2 抵亏 / used</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>所得税 income y=2 / Income income y=2 到期核销 / expired</t>
+          <t xml:space="preserve">所得税 income y=2 / Income income y=2 新生亏损 / generated</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>所得税 income y=2 / Income income y=2 税额 / tax</t>
+          <t xml:space="preserve">所得税 income y=2 / Income income y=2 到期核销 / expired</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>119092.87610620132 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>所得税 income y=3 / Income income y=3 税基 / base</t>
+          <t xml:space="preserve">所得税 income y=2 / Income income y=2 税额 / tax</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>476460.0 CNY</t>
+          <t xml:space="preserve">119092.87610620132 CNY</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>所得税 income y=3 / Income income y=3 抵亏 / used</t>
+          <t xml:space="preserve">所得税 income y=3 / Income income y=3 税基 / base</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">476460.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>所得税 income y=3 / Income income y=3 新生亏损 / generated</t>
+          <t xml:space="preserve">所得税 income y=3 / Income income y=3 抵亏 / used</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>所得税 income y=3 / Income income y=3 到期核销 / expired</t>
+          <t xml:space="preserve">所得税 income y=3 / Income income y=3 新生亏损 / generated</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>所得税 income y=3 / Income income y=3 税额 / tax</t>
+          <t xml:space="preserve">所得税 income y=3 / Income income y=3 到期核销 / expired</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>119115.00000000664 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>计税折旧 income pv_system y=2 / Depreciation income pv_system y=2</t>
+          <t xml:space="preserve">所得税 income y=3 / Income income y=3 税额 / tax</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>30000.0 CNY</t>
+          <t xml:space="preserve">119115.00000000664 CNY</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>计税折旧 income pv_system y=3 / Depreciation income pv_system y=3</t>
+          <t xml:space="preserve">计税折旧 income upfront_capex_net:pv_system y=2 / Depreciation income upfront_capex_net:pv_system y=2</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>30000.0 CNY</t>
+          <t xml:space="preserve">30000.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>亏损余额 income v0 y=2 (可用至y=7) / Loss balance</t>
+          <t xml:space="preserve">计税折旧 income upfront_capex_net:pv_system y=3 / Depreciation income upfront_capex_net:pv_system y=3</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">30000.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>亏损余额 income v0 y=3 (可用至y=7) / Loss balance</t>
+          <t xml:space="preserve">亏损余额 income v0 y=2 (可用至y=7) / Loss balance</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>亏损余额 income v1 y=3 (可用至y=8) / Loss balance</t>
+          <t xml:space="preserve">亏损余额 income v0 y=3 (可用至y=7) / Loss balance</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>0.0 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>净现值 NPV / NPV</t>
+          <t xml:space="preserve">亏损余额 income v1 y=3 (可用至y=8) / Loss balance</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>46532.2713683926116308489560 CNY</t>
+          <t xml:space="preserve">0.0 CNY</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>内部收益率 IRR / IRR</t>
+          <t xml:space="preserve">净现值 NPV / NPV</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>0.11632899562309858 / normal</t>
+          <t xml:space="preserve">46532.2713683926116308489560 CNY</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>静态回收期 / static payback</t>
+          <t xml:space="preserve">内部收益率 IRR / IRR</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2.564097557315646 year / recovered</t>
+          <t xml:space="preserve">0.11632899562309858 / normal</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>动态回收期 / dynamic payback</t>
+          <t xml:space="preserve">静态回收期 / static payback</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2.8523668375110995 year / recovered</t>
+          <t xml:space="preserve">2.564097557315646 year / recovered</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t xml:space="preserve">动态回收期 / dynamic payback</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2.8523668375110995 year / recovered</t>
         </is>
       </c>
     </row>

</xml_diff>